<commit_message>
Add daily test page + learning log: 2026-09-13
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y98"/>
+  <dimension ref="A1:Y99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12000,6 +12000,123 @@
         </is>
       </c>
     </row>
+    <row r="99" ht="60" customHeight="1">
+      <c r="A99" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B99" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C99" s="9" t="inlineStr">
+        <is>
+          <t>능력·공손 조동사</t>
+        </is>
+      </c>
+      <c r="D99" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: can / could — 능력과 공손</t>
+        </is>
+      </c>
+      <c r="E99" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F99" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G99" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H99" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I99" s="9" t="inlineStr">
+        <is>
+          <t>shofar</t>
+        </is>
+      </c>
+      <c r="J99" s="9" t="inlineStr">
+        <is>
+          <t>So, have you ever heard of a shofar? It's this ancient horn instrument made from a ram's horn that Jewish people have used for thousands of years. They blow it during important religious holidays like Rosh Hashanah to signal special moments. It's actually a really meaningful tradition that connects modern Judaism to ancient history.</t>
+        </is>
+      </c>
+      <c r="K99" s="9" t="inlineStr">
+        <is>
+          <t>signal — 신호를 보내다, 알리다; tradition — 전통</t>
+        </is>
+      </c>
+      <c r="L99" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M99" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N99" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O99" s="9" t="inlineStr">
+        <is>
+          <t>문장 강세와 리듬</t>
+        </is>
+      </c>
+      <c r="P99" s="9" t="inlineStr">
+        <is>
+          <t>내용어(명사·동사·형용사)는 강하게, 기능어(관사·전치사)는 약하게</t>
+        </is>
+      </c>
+      <c r="Q99" s="9" t="inlineStr">
+        <is>
+          <t>I WANT to GO to the STORE | She's WORKING on a NEW project</t>
+        </is>
+      </c>
+      <c r="R99" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S99" s="9" t="inlineStr"/>
+      <c r="T99" s="9" t="inlineStr"/>
+      <c r="U99" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V99" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W99" s="9" t="inlineStr">
+        <is>
+          <t>invest</t>
+        </is>
+      </c>
+      <c r="X99" s="9" t="inlineStr">
+        <is>
+          <t>투자하다</t>
+        </is>
+      </c>
+      <c r="Y99" s="9" t="inlineStr">
+        <is>
+          <t>중세에 왕이 신하에게 땅을 수여할 때 옷(vestis)을 입혀 권한 부여</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-14
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y99"/>
+  <dimension ref="A1:Y100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12117,6 +12117,123 @@
         </is>
       </c>
     </row>
+    <row r="100" ht="60" customHeight="1">
+      <c r="A100" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B100" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C100" s="9" t="inlineStr">
+        <is>
+          <t>실현 가능한 조건문</t>
+        </is>
+      </c>
+      <c r="D100" s="9" t="inlineStr">
+        <is>
+          <t>First Conditional</t>
+        </is>
+      </c>
+      <c r="E100" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F100" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G100" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H100" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I100" s="9" t="inlineStr">
+        <is>
+          <t>empirical</t>
+        </is>
+      </c>
+      <c r="J100" s="9" t="inlineStr">
+        <is>
+          <t>So we've been collecting data from our research for five years now, and all the results are empirical—meaning they're based on actual observations and experiments, not just theories. Our team can actually prove everything we found because we tested it ourselves. That's why companies really trust empirical evidence when they're making important business decisions.</t>
+        </is>
+      </c>
+      <c r="K100" s="9" t="inlineStr">
+        <is>
+          <t>empirical — 실증적인, 경험·관찰에 기반한; evidence — 증거, 근거</t>
+        </is>
+      </c>
+      <c r="L100" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M100" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N100" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O100" s="9" t="inlineStr">
+        <is>
+          <t>억양: 의문문</t>
+        </is>
+      </c>
+      <c r="P100" s="9" t="inlineStr">
+        <is>
+          <t>Yes/No 질문은 끝이 올라가고 ↗, Wh- 질문은 끝이 내려감 ↘</t>
+        </is>
+      </c>
+      <c r="Q100" s="9" t="inlineStr">
+        <is>
+          <t>Are you READY? ↗ | Where are you GOING? ↘ | Did you SEE it? ↗</t>
+        </is>
+      </c>
+      <c r="R100" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S100" s="9" t="inlineStr"/>
+      <c r="T100" s="9" t="inlineStr"/>
+      <c r="U100" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V100" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W100" s="9" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="X100" s="9" t="inlineStr">
+        <is>
+          <t>위험, 위험을 감수하다</t>
+        </is>
+      </c>
+      <c r="Y100" s="9" t="inlineStr">
+        <is>
+          <t>항해 중 암초 근처를 항행하는 위험에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-15
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y100"/>
+  <dimension ref="A1:Y101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12234,6 +12234,123 @@
         </is>
       </c>
     </row>
+    <row r="101" ht="60" customHeight="1">
+      <c r="A101" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B101" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C101" s="9" t="inlineStr">
+        <is>
+          <t>수동태</t>
+        </is>
+      </c>
+      <c r="D101" s="9" t="inlineStr">
+        <is>
+          <t>Passive Voice</t>
+        </is>
+      </c>
+      <c r="E101" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F101" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G101" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H101" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I101" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Pygmalion</t>
+        </is>
+      </c>
+      <c r="J101" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a classic story called Pygmalion, and we're going to focus on eight different uses of the word 'round'. It's a great way to learn how one simple word can have many different meanings in English. So stick around for five minutes, and by the end, you'll understand how to use 'round' naturally in conversation.</t>
+        </is>
+      </c>
+      <c r="K101" s="9" t="inlineStr">
+        <is>
+          <t>stick around — 계속 있다, 머물다; focus on — ~에 초점을 맞추다</t>
+        </is>
+      </c>
+      <c r="L101" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M101" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N101" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O101" s="9" t="inlineStr">
+        <is>
+          <t>r vs l 구분</t>
+        </is>
+      </c>
+      <c r="P101" s="9" t="inlineStr">
+        <is>
+          <t>r은 혀를 말아 입천장에 닿지 않게, l은 혀끝을 윗잇몸에 확실히 댐</t>
+        </is>
+      </c>
+      <c r="Q101" s="9" t="inlineStr">
+        <is>
+          <t>really /ríːli/ | rally /réli/ | river /rívər/ | liver /lívər/</t>
+        </is>
+      </c>
+      <c r="R101" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S101" s="9" t="inlineStr"/>
+      <c r="T101" s="9" t="inlineStr"/>
+      <c r="U101" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V101" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W101" s="9" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
+      <c r="X101" s="9" t="inlineStr">
+        <is>
+          <t>예산</t>
+        </is>
+      </c>
+      <c r="Y101" s="9" t="inlineStr">
+        <is>
+          <t>재무장관이 예산서를 담은 가죽 가방(bougette)을 들고 의회에 출석한 데서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-16
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y101"/>
+  <dimension ref="A1:Y102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12351,6 +12351,123 @@
         </is>
       </c>
     </row>
+    <row r="102" ht="60" customHeight="1">
+      <c r="A102" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B102" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C102" s="9" t="inlineStr">
+        <is>
+          <t>관사</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="inlineStr">
+        <is>
+          <t>Articles: a / an / the</t>
+        </is>
+      </c>
+      <c r="E102" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F102" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G102" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H102" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I102" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Pygmalion</t>
+        </is>
+      </c>
+      <c r="J102" s="9" t="inlineStr">
+        <is>
+          <t>Today we're exploring a classic story called Pygmalion, where we'll learn eight different uses of the word 'round'. The story takes place in ancient Greece, and it's all about an artist who falls in love with his own sculpture. As we go through the narrative, you'll pick up how 'round' works in various contexts, which is really useful for everyday conversation.</t>
+        </is>
+      </c>
+      <c r="K102" s="9" t="inlineStr">
+        <is>
+          <t>narrative — 이야기, 내러티브; sculpture — 조각상, 조각 작품</t>
+        </is>
+      </c>
+      <c r="L102" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M102" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N102" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O102" s="9" t="inlineStr">
+        <is>
+          <t>f vs p 구분</t>
+        </is>
+      </c>
+      <c r="P102" s="9" t="inlineStr">
+        <is>
+          <t>f는 윗니를 아랫입술에 대고 바람, p는 두 입술로 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q102" s="9" t="inlineStr">
+        <is>
+          <t>food /fuːd/ | pool /puːl/ | fee /fiː/ | pea /piː/</t>
+        </is>
+      </c>
+      <c r="R102" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S102" s="9" t="inlineStr"/>
+      <c r="T102" s="9" t="inlineStr"/>
+      <c r="U102" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V102" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W102" s="9" t="inlineStr">
+        <is>
+          <t>magazine</t>
+        </is>
+      </c>
+      <c r="X102" s="9" t="inlineStr">
+        <is>
+          <t>잡지, 탄창</t>
+        </is>
+      </c>
+      <c r="Y102" s="9" t="inlineStr">
+        <is>
+          <t>지식·정보를 저장해 두는 '창고'라는 의미로 출판물에 사용됨</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-17
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y102"/>
+  <dimension ref="A1:Y103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12468,6 +12468,123 @@
         </is>
       </c>
     </row>
+    <row r="103" ht="60" customHeight="1">
+      <c r="A103" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B103" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C103" s="9" t="inlineStr">
+        <is>
+          <t>강조 도치</t>
+        </is>
+      </c>
+      <c r="D103" s="9" t="inlineStr">
+        <is>
+          <t>Inversion for Emphasis</t>
+        </is>
+      </c>
+      <c r="E103" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F103" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G103" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H103" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I103" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Pygmalion</t>
+        </is>
+      </c>
+      <c r="J103" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore a classic story called Pygmalion and learn different ways to use the word 'round'. This story is all about an artist who falls in love with his own creation. As we go through the tale, you'll pick up eight useful meanings of 'round' that you can use in everyday conversations and at work.</t>
+        </is>
+      </c>
+      <c r="K103" s="9" t="inlineStr">
+        <is>
+          <t>creation — 창작물, 작품; pick up — (언어나 기술을) 배우다, 습득하다</t>
+        </is>
+      </c>
+      <c r="L103" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M103" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N103" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O103" s="9" t="inlineStr">
+        <is>
+          <t>v vs b 구분</t>
+        </is>
+      </c>
+      <c r="P103" s="9" t="inlineStr">
+        <is>
+          <t>v는 윗니를 아랫입술에 대고 진동, b는 두 입술로 막아 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q103" s="9" t="inlineStr">
+        <is>
+          <t>very /véri/ | berry /béri/ | vest /vest/ | best /best/</t>
+        </is>
+      </c>
+      <c r="R103" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S103" s="9" t="inlineStr"/>
+      <c r="T103" s="9" t="inlineStr"/>
+      <c r="U103" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V103" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W103" s="9" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="X103" s="9" t="inlineStr">
+        <is>
+          <t>후보자</t>
+        </is>
+      </c>
+      <c r="Y103" s="9" t="inlineStr">
+        <is>
+          <t>로마 선거 출마자는 순결을 상징하는 흰 토가를 입었음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-18
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y103"/>
+  <dimension ref="A1:Y104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12585,6 +12585,123 @@
         </is>
       </c>
     </row>
+    <row r="104" ht="60" customHeight="1">
+      <c r="A104" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B104" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C104" s="9" t="inlineStr">
+        <is>
+          <t>과거완료</t>
+        </is>
+      </c>
+      <c r="D104" s="9" t="inlineStr">
+        <is>
+          <t>Past Perfect Tense</t>
+        </is>
+      </c>
+      <c r="E104" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F104" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G104" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H104" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I104" s="9" t="inlineStr">
+        <is>
+          <t>churlish</t>
+        </is>
+      </c>
+      <c r="J104" s="9" t="inlineStr">
+        <is>
+          <t>You know, my boss made some really churlish comments about my project yesterday. I was pretty shocked, honestly. Instead of giving constructive feedback, he just complained without offering any helpful suggestions. I think he needs to work on his communication skills.</t>
+        </is>
+      </c>
+      <c r="K104" s="9" t="inlineStr">
+        <is>
+          <t>churlish — 무례한, 버릇없는; constructive feedback — 건설적인 피드백</t>
+        </is>
+      </c>
+      <c r="L104" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M104" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N104" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O104" s="9" t="inlineStr">
+        <is>
+          <t>th 유성음 /ð/</t>
+        </is>
+      </c>
+      <c r="P104" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 목소리 진동</t>
+        </is>
+      </c>
+      <c r="Q104" s="9" t="inlineStr">
+        <is>
+          <t>the /ðə/ | this /ðɪs/ | that /ðæt/ | mother /mʌðər/</t>
+        </is>
+      </c>
+      <c r="R104" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S104" s="9" t="inlineStr"/>
+      <c r="T104" s="9" t="inlineStr"/>
+      <c r="U104" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V104" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W104" s="9" t="inlineStr">
+        <is>
+          <t>serendipity</t>
+        </is>
+      </c>
+      <c r="X104" s="9" t="inlineStr">
+        <is>
+          <t>뜻밖의 행운</t>
+        </is>
+      </c>
+      <c r="Y104" s="9" t="inlineStr">
+        <is>
+          <t>세 왕자가 우연히 훌륭한 발견을 하는 동화에서 Horace Walpole이 만든 단어</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-19
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y104"/>
+  <dimension ref="A1:Y105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12702,6 +12702,123 @@
         </is>
       </c>
     </row>
+    <row r="105" ht="60" customHeight="1">
+      <c r="A105" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B105" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C105" s="9" t="inlineStr">
+        <is>
+          <t>의무·충고 조동사</t>
+        </is>
+      </c>
+      <c r="D105" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: should / ought to / had better</t>
+        </is>
+      </c>
+      <c r="E105" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F105" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G105" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H105" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I105" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Pride and Prejudice</t>
+        </is>
+      </c>
+      <c r="J105" s="9" t="inlineStr">
+        <is>
+          <t>Have you ever noticed how the word 'look' has so many different meanings in English? In Pride and Prejudice, characters constantly look at each other—sometimes they look down on others, sometimes they look forward to meeting someone new. Understanding these different uses of 'look' will really improve your daily conversations and help you communicate more naturally.</t>
+        </is>
+      </c>
+      <c r="K105" s="9" t="inlineStr">
+        <is>
+          <t>look down on — ~을 무시하다/깔보다; look forward to — ~을 기대하다</t>
+        </is>
+      </c>
+      <c r="L105" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M105" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N105" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O105" s="9" t="inlineStr">
+        <is>
+          <t>th 무성음 /θ/</t>
+        </is>
+      </c>
+      <c r="P105" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 바람만 내보냄</t>
+        </is>
+      </c>
+      <c r="Q105" s="9" t="inlineStr">
+        <is>
+          <t>think /θɪŋk/ | three /θriː/ | health /helθ/ | month /mʌnθ/</t>
+        </is>
+      </c>
+      <c r="R105" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S105" s="9" t="inlineStr"/>
+      <c r="T105" s="9" t="inlineStr"/>
+      <c r="U105" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V105" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W105" s="9" t="inlineStr">
+        <is>
+          <t>berserk</t>
+        </is>
+      </c>
+      <c r="X105" s="9" t="inlineStr">
+        <is>
+          <t>극도로 흥분한, 폭주하는</t>
+        </is>
+      </c>
+      <c r="Y105" s="9" t="inlineStr">
+        <is>
+          <t>전투에서 곰 가죽을 입고 광분하던 바이킹 전사에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-20
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y105"/>
+  <dimension ref="A1:Y106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12819,6 +12819,123 @@
         </is>
       </c>
     </row>
+    <row r="106" ht="60" customHeight="1">
+      <c r="A106" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B106" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C106" s="9" t="inlineStr">
+        <is>
+          <t>가정법 과거</t>
+        </is>
+      </c>
+      <c r="D106" s="9" t="inlineStr">
+        <is>
+          <t>Second Conditional</t>
+        </is>
+      </c>
+      <c r="E106" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F106" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G106" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H106" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I106" s="9" t="inlineStr">
+        <is>
+          <t>volition</t>
+        </is>
+      </c>
+      <c r="J106" s="9" t="inlineStr">
+        <is>
+          <t>So, Sarah quit her job last month. Was it because the company forced her to leave? No, actually she left of her own volition. She just decided it was time for a change. Sometimes people need to make their own choices, you know?</t>
+        </is>
+      </c>
+      <c r="K106" s="9" t="inlineStr">
+        <is>
+          <t>volition — 자발적인 선택/결정 능력; of one's own volition — 자발적으로, 스스로의 의지로</t>
+        </is>
+      </c>
+      <c r="L106" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M106" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N106" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O106" s="9" t="inlineStr">
+        <is>
+          <t>짧은 모음 vs 긴 모음</t>
+        </is>
+      </c>
+      <c r="P106" s="9" t="inlineStr">
+        <is>
+          <t>ship /ɪ/ vs sheep /iː/ — 입 모양과 길이 모두 다름</t>
+        </is>
+      </c>
+      <c r="Q106" s="9" t="inlineStr">
+        <is>
+          <t>ship /ʃɪp/ | sheep /ʃiːp/ | hit /hɪt/ | heat /hiːt/</t>
+        </is>
+      </c>
+      <c r="R106" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S106" s="9" t="inlineStr"/>
+      <c r="T106" s="9" t="inlineStr"/>
+      <c r="U106" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V106" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W106" s="9" t="inlineStr">
+        <is>
+          <t>boycott</t>
+        </is>
+      </c>
+      <c r="X106" s="9" t="inlineStr">
+        <is>
+          <t>불매운동, 거부하다</t>
+        </is>
+      </c>
+      <c r="Y106" s="9" t="inlineStr">
+        <is>
+          <t>1880년 소작인들이 Boycott을 집단 거부한 사건에서 단어화</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-21
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y106"/>
+  <dimension ref="A1:Y107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12936,6 +12936,123 @@
         </is>
       </c>
     </row>
+    <row r="107" ht="60" customHeight="1">
+      <c r="A107" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B107" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C107" s="9" t="inlineStr">
+        <is>
+          <t>간접화법</t>
+        </is>
+      </c>
+      <c r="D107" s="9" t="inlineStr">
+        <is>
+          <t>Reported Speech</t>
+        </is>
+      </c>
+      <c r="E107" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F107" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G107" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H107" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I107" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Pride and Prejudice</t>
+        </is>
+      </c>
+      <c r="J107" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at Jane Austen's Pride and Prejudice, one of the most famous novels ever written. In this story, we'll explore how the word 'look' is used in different ways throughout the narrative. By the end of this five-minute lesson, you'll understand eleven different meanings of 'look' and how to use them naturally in everyday conversation.</t>
+        </is>
+      </c>
+      <c r="K107" s="9" t="inlineStr">
+        <is>
+          <t>explore — 탐구하다, 조사하다; narrative — 이야기, 서술</t>
+        </is>
+      </c>
+      <c r="L107" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M107" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N107" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O107" s="9" t="inlineStr">
+        <is>
+          <t>어말 자음 탈락 방지</t>
+        </is>
+      </c>
+      <c r="P107" s="9" t="inlineStr">
+        <is>
+          <t>한국어는 받침 뒤 모음을 붙이는 경향 — 마지막 자음만 닫고 끝내기</t>
+        </is>
+      </c>
+      <c r="Q107" s="9" t="inlineStr">
+        <is>
+          <t>fact /fækt/ | next /nekst/ | helped /helpt/ | asked /æskt/</t>
+        </is>
+      </c>
+      <c r="R107" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S107" s="9" t="inlineStr"/>
+      <c r="T107" s="9" t="inlineStr"/>
+      <c r="U107" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V107" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W107" s="9" t="inlineStr">
+        <is>
+          <t>mentor</t>
+        </is>
+      </c>
+      <c r="X107" s="9" t="inlineStr">
+        <is>
+          <t>멘토, 스승</t>
+        </is>
+      </c>
+      <c r="Y107" s="9" t="inlineStr">
+        <is>
+          <t>오디세우스가 트로이 전쟁 중 아들 텔레마코스 교육을 맡긴 현자의 이름에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-22
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y107"/>
+  <dimension ref="A1:Y108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13053,6 +13053,123 @@
         </is>
       </c>
     </row>
+    <row r="108" ht="60" customHeight="1">
+      <c r="A108" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B108" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C108" s="9" t="inlineStr">
+        <is>
+          <t>동명사 vs 부정사</t>
+        </is>
+      </c>
+      <c r="D108" s="9" t="inlineStr">
+        <is>
+          <t>Gerunds vs Infinitives</t>
+        </is>
+      </c>
+      <c r="E108" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F108" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G108" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H108" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I108" s="9" t="inlineStr">
+        <is>
+          <t>nemesis</t>
+        </is>
+      </c>
+      <c r="J108" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K108" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L108" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M108" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N108" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O108" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 명사</t>
+        </is>
+      </c>
+      <c r="P108" s="9" t="inlineStr">
+        <is>
+          <t>명사는 보통 첫 음절 강세 — REcord, PROtest, PERmit</t>
+        </is>
+      </c>
+      <c r="Q108" s="9" t="inlineStr">
+        <is>
+          <t>REcord | PROtest | PERmit | CONtent</t>
+        </is>
+      </c>
+      <c r="R108" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S108" s="9" t="inlineStr"/>
+      <c r="T108" s="9" t="inlineStr"/>
+      <c r="U108" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V108" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W108" s="9" t="inlineStr">
+        <is>
+          <t>rival</t>
+        </is>
+      </c>
+      <c r="X108" s="9" t="inlineStr">
+        <is>
+          <t>경쟁자</t>
+        </is>
+      </c>
+      <c r="Y108" s="9" t="inlineStr">
+        <is>
+          <t>같은 강(rivus) 물을 사용하는 이웃 사이의 경쟁 관계에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-23
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y108"/>
+  <dimension ref="A1:Y109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13170,6 +13170,123 @@
         </is>
       </c>
     </row>
+    <row r="109" ht="60" customHeight="1">
+      <c r="A109" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B109" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C109" s="9" t="inlineStr">
+        <is>
+          <t>가정법 현재 (요구·제안 구문)</t>
+        </is>
+      </c>
+      <c r="D109" s="9" t="inlineStr">
+        <is>
+          <t>Subjunctive Mood</t>
+        </is>
+      </c>
+      <c r="E109" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F109" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G109" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H109" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I109" s="9" t="inlineStr">
+        <is>
+          <t>compendious</t>
+        </is>
+      </c>
+      <c r="J109" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K109" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L109" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M109" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N109" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O109" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 동사</t>
+        </is>
+      </c>
+      <c r="P109" s="9" t="inlineStr">
+        <is>
+          <t>동사는 보통 두 번째 음절 강세 — reCORD, proTEST, perMIT</t>
+        </is>
+      </c>
+      <c r="Q109" s="9" t="inlineStr">
+        <is>
+          <t>reCORD | proTEST | perMIT | conTENT</t>
+        </is>
+      </c>
+      <c r="R109" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S109" s="9" t="inlineStr"/>
+      <c r="T109" s="9" t="inlineStr"/>
+      <c r="U109" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V109" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W109" s="9" t="inlineStr">
+        <is>
+          <t>travel</t>
+        </is>
+      </c>
+      <c r="X109" s="9" t="inlineStr">
+        <is>
+          <t>여행하다</t>
+        </is>
+      </c>
+      <c r="Y109" s="9" t="inlineStr">
+        <is>
+          <t>중세 여행이 고문(tripalium)처럼 고달팠던 데서 travail(고통)과 동근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-24
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y109"/>
+  <dimension ref="A1:Y110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13287,6 +13287,123 @@
         </is>
       </c>
     </row>
+    <row r="110" ht="60" customHeight="1">
+      <c r="A110" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B110" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C110" s="9" t="inlineStr">
+        <is>
+          <t>미래 표현 3가지</t>
+        </is>
+      </c>
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>Future Tenses: will / going to / present continuous</t>
+        </is>
+      </c>
+      <c r="E110" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F110" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G110" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H110" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I110" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Pride and Prejudice</t>
+        </is>
+      </c>
+      <c r="J110" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K110" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L110" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M110" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N110" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O110" s="9" t="inlineStr">
+        <is>
+          <t>-ed 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P110" s="9" t="inlineStr">
+        <is>
+          <t>/t/: 무성음 뒤 | /d/: 유성음 뒤 | /ɪd/: t·d로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q110" s="9" t="inlineStr">
+        <is>
+          <t>worked /wɜːrkt/ | called /kɔːld/ | wanted /wɒntɪd/ | needed /niːdɪd/</t>
+        </is>
+      </c>
+      <c r="R110" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S110" s="9" t="inlineStr"/>
+      <c r="T110" s="9" t="inlineStr"/>
+      <c r="U110" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V110" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W110" s="9" t="inlineStr">
+        <is>
+          <t>enthusiasm</t>
+        </is>
+      </c>
+      <c r="X110" s="9" t="inlineStr">
+        <is>
+          <t>열정, 열의</t>
+        </is>
+      </c>
+      <c r="Y110" s="9" t="inlineStr">
+        <is>
+          <t>en(안에) + theos(신) → 신에게 감화받은 열정 상태</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-25
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y110"/>
+  <dimension ref="A1:Y111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13404,6 +13404,123 @@
         </is>
       </c>
     </row>
+    <row r="111" ht="60" customHeight="1">
+      <c r="A111" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B111" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C111" s="9" t="inlineStr">
+        <is>
+          <t>의무·필요 조동사</t>
+        </is>
+      </c>
+      <c r="D111" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: must / have to / need to</t>
+        </is>
+      </c>
+      <c r="E111" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F111" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G111" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H111" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I111" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Robin Hood</t>
+        </is>
+      </c>
+      <c r="J111" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K111" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L111" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M111" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N111" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O111" s="9" t="inlineStr">
+        <is>
+          <t>-s/-es 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P111" s="9" t="inlineStr">
+        <is>
+          <t>/ s/: 무성음 뒤 | /z/: 유성음 뒤 | /ɪz/: s·z·ch·sh로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q111" s="9" t="inlineStr">
+        <is>
+          <t>books /bʊks/ | dogs /dɒgz/ | watches /wɒtʃɪz/ | buses /bʌsɪz/</t>
+        </is>
+      </c>
+      <c r="R111" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S111" s="9" t="inlineStr"/>
+      <c r="T111" s="9" t="inlineStr"/>
+      <c r="U111" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V111" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W111" s="9" t="inlineStr">
+        <is>
+          <t>lucid</t>
+        </is>
+      </c>
+      <c r="X111" s="9" t="inlineStr">
+        <is>
+          <t>명확한, 이해하기 쉬운</t>
+        </is>
+      </c>
+      <c r="Y111" s="9" t="inlineStr">
+        <is>
+          <t>lux(빛)과 동근 → 명확하고 투명한 사고</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-26
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y111"/>
+  <dimension ref="A1:Y112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13521,6 +13521,123 @@
         </is>
       </c>
     </row>
+    <row r="112" ht="60" customHeight="1">
+      <c r="A112" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B112" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C112" s="9" t="inlineStr">
+        <is>
+          <t>가정법 과거완료·혼합</t>
+        </is>
+      </c>
+      <c r="D112" s="9" t="inlineStr">
+        <is>
+          <t>Third Conditional &amp; Mixed Conditionals</t>
+        </is>
+      </c>
+      <c r="E112" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F112" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G112" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H112" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I112" s="9" t="inlineStr">
+        <is>
+          <t>confabulate</t>
+        </is>
+      </c>
+      <c r="J112" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K112" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L112" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M112" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N112" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O112" s="9" t="inlineStr">
+        <is>
+          <t>연음 (Linking)</t>
+        </is>
+      </c>
+      <c r="P112" s="9" t="inlineStr">
+        <is>
+          <t>자음으로 끝나는 단어 + 모음으로 시작하는 단어는 이어서 발음</t>
+        </is>
+      </c>
+      <c r="Q112" s="9" t="inlineStr">
+        <is>
+          <t>pick it up → pi-ki-tup | turn it on → tur-ni-ton | look at it → loo-ka-tit</t>
+        </is>
+      </c>
+      <c r="R112" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S112" s="9" t="inlineStr"/>
+      <c r="T112" s="9" t="inlineStr"/>
+      <c r="U112" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V112" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W112" s="9" t="inlineStr">
+        <is>
+          <t>colleague</t>
+        </is>
+      </c>
+      <c r="X112" s="9" t="inlineStr">
+        <is>
+          <t>동료</t>
+        </is>
+      </c>
+      <c r="Y112" s="9" t="inlineStr">
+        <is>
+          <t>col(함께) + legare(선택하다/보내다) → 같이 선발된 동료</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-27
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y112"/>
+  <dimension ref="A1:Y113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13638,6 +13638,123 @@
         </is>
       </c>
     </row>
+    <row r="113" ht="60" customHeight="1">
+      <c r="A113" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B113" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C113" s="9" t="inlineStr">
+        <is>
+          <t>관계절</t>
+        </is>
+      </c>
+      <c r="D113" s="9" t="inlineStr">
+        <is>
+          <t>Relative Clauses: defining vs non-defining</t>
+        </is>
+      </c>
+      <c r="E113" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F113" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G113" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H113" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I113" s="9" t="inlineStr">
+        <is>
+          <t>bellwether</t>
+        </is>
+      </c>
+      <c r="J113" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K113" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L113" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M113" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N113" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O113" s="9" t="inlineStr">
+        <is>
+          <t>약화 (Reduction)</t>
+        </is>
+      </c>
+      <c r="P113" s="9" t="inlineStr">
+        <is>
+          <t>기능어(of·to·for·and·at)는 빠르게 약화 — /ə/ 로 줄어듦</t>
+        </is>
+      </c>
+      <c r="Q113" s="9" t="inlineStr">
+        <is>
+          <t>cup of tea → cupə tea | a lot of → ə lɒtə | want to → wanna</t>
+        </is>
+      </c>
+      <c r="R113" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S113" s="9" t="inlineStr"/>
+      <c r="T113" s="9" t="inlineStr"/>
+      <c r="U113" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V113" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W113" s="9" t="inlineStr">
+        <is>
+          <t>quarantine</t>
+        </is>
+      </c>
+      <c r="X113" s="9" t="inlineStr">
+        <is>
+          <t>격리, 검역</t>
+        </is>
+      </c>
+      <c r="Y113" s="9" t="inlineStr">
+        <is>
+          <t>14세기 흑사병 때 선박을 40일간 격리한 베네치아 방역 정책에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-28
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y113"/>
+  <dimension ref="A1:Y114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13755,6 +13755,123 @@
         </is>
       </c>
     </row>
+    <row r="114" ht="60" customHeight="1">
+      <c r="A114" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B114" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C114" s="9" t="inlineStr">
+        <is>
+          <t>시간 전치사</t>
+        </is>
+      </c>
+      <c r="D114" s="9" t="inlineStr">
+        <is>
+          <t>Prepositions of Time: at / in / on / by</t>
+        </is>
+      </c>
+      <c r="E114" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F114" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G114" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H114" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I114" s="9" t="inlineStr">
+        <is>
+          <t>fungible</t>
+        </is>
+      </c>
+      <c r="J114" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K114" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L114" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M114" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N114" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O114" s="9" t="inlineStr">
+        <is>
+          <t>문장 강세와 리듬</t>
+        </is>
+      </c>
+      <c r="P114" s="9" t="inlineStr">
+        <is>
+          <t>내용어(명사·동사·형용사)는 강하게, 기능어(관사·전치사)는 약하게</t>
+        </is>
+      </c>
+      <c r="Q114" s="9" t="inlineStr">
+        <is>
+          <t>I WANT to GO to the STORE | She's WORKING on a NEW project</t>
+        </is>
+      </c>
+      <c r="R114" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S114" s="9" t="inlineStr"/>
+      <c r="T114" s="9" t="inlineStr"/>
+      <c r="U114" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V114" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W114" s="9" t="inlineStr">
+        <is>
+          <t>clue</t>
+        </is>
+      </c>
+      <c r="X114" s="9" t="inlineStr">
+        <is>
+          <t>단서, 실마리</t>
+        </is>
+      </c>
+      <c r="Y114" s="9" t="inlineStr">
+        <is>
+          <t>그리스 신화에서 테세우스가 미로를 탈출할 때 아리아드네의 실(clew)에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-29
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y114"/>
+  <dimension ref="A1:Y115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13872,6 +13872,123 @@
         </is>
       </c>
     </row>
+    <row r="115" ht="60" customHeight="1">
+      <c r="A115" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B115" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C115" s="9" t="inlineStr">
+        <is>
+          <t>생략과 대용</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="inlineStr">
+        <is>
+          <t>Ellipsis and Substitution</t>
+        </is>
+      </c>
+      <c r="E115" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F115" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G115" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H115" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I115" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Robin Hood</t>
+        </is>
+      </c>
+      <c r="J115" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K115" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L115" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M115" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N115" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O115" s="9" t="inlineStr">
+        <is>
+          <t>억양: 의문문</t>
+        </is>
+      </c>
+      <c r="P115" s="9" t="inlineStr">
+        <is>
+          <t>Yes/No 질문은 끝이 올라가고 ↗, Wh- 질문은 끝이 내려감 ↘</t>
+        </is>
+      </c>
+      <c r="Q115" s="9" t="inlineStr">
+        <is>
+          <t>Are you READY? ↗ | Where are you GOING? ↘ | Did you SEE it? ↗</t>
+        </is>
+      </c>
+      <c r="R115" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S115" s="9" t="inlineStr"/>
+      <c r="T115" s="9" t="inlineStr"/>
+      <c r="U115" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V115" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W115" s="9" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="X115" s="9" t="inlineStr">
+        <is>
+          <t>급여</t>
+        </is>
+      </c>
+      <c r="Y115" s="9" t="inlineStr">
+        <is>
+          <t>로마 병사의 소금 급여에서. '소금값 못하는 사람'이라는 표현도 여기서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-30
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y115"/>
+  <dimension ref="A1:Y116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13989,6 +13989,123 @@
         </is>
       </c>
     </row>
+    <row r="116" ht="60" customHeight="1">
+      <c r="A116" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B116" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C116" s="9" t="inlineStr">
+        <is>
+          <t>단순현재 vs 현재진행</t>
+        </is>
+      </c>
+      <c r="D116" s="9" t="inlineStr">
+        <is>
+          <t>Present Simple vs Present Continuous</t>
+        </is>
+      </c>
+      <c r="E116" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F116" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G116" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H116" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I116" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Robin Hood</t>
+        </is>
+      </c>
+      <c r="J116" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K116" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L116" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M116" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N116" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O116" s="9" t="inlineStr">
+        <is>
+          <t>r vs l 구분</t>
+        </is>
+      </c>
+      <c r="P116" s="9" t="inlineStr">
+        <is>
+          <t>r은 혀를 말아 입천장에 닿지 않게, l은 혀끝을 윗잇몸에 확실히 댐</t>
+        </is>
+      </c>
+      <c r="Q116" s="9" t="inlineStr">
+        <is>
+          <t>really /ríːli/ | rally /réli/ | river /rívər/ | liver /lívər/</t>
+        </is>
+      </c>
+      <c r="R116" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S116" s="9" t="inlineStr"/>
+      <c r="T116" s="9" t="inlineStr"/>
+      <c r="U116" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V116" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W116" s="9" t="inlineStr">
+        <is>
+          <t>sincere</t>
+        </is>
+      </c>
+      <c r="X116" s="9" t="inlineStr">
+        <is>
+          <t>진실한, 진심 어린</t>
+        </is>
+      </c>
+      <c r="Y116" s="9" t="inlineStr">
+        <is>
+          <t>로마 조각가가 결함을 밀랍으로 숨겼는데, 최고 작품은 밀랍 없이(sine cera) 완성됨</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-01
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y116"/>
+  <dimension ref="A1:Y117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14106,6 +14106,123 @@
         </is>
       </c>
     </row>
+    <row r="117" ht="60" customHeight="1">
+      <c r="A117" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B117" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C117" s="9" t="inlineStr">
+        <is>
+          <t>구동사 (비즈니스)</t>
+        </is>
+      </c>
+      <c r="D117" s="9" t="inlineStr">
+        <is>
+          <t>Phrasal Verbs – Business Context</t>
+        </is>
+      </c>
+      <c r="E117" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F117" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G117" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H117" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I117" s="9" t="inlineStr">
+        <is>
+          <t>slew</t>
+        </is>
+      </c>
+      <c r="J117" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K117" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L117" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M117" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N117" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O117" s="9" t="inlineStr">
+        <is>
+          <t>f vs p 구분</t>
+        </is>
+      </c>
+      <c r="P117" s="9" t="inlineStr">
+        <is>
+          <t>f는 윗니를 아랫입술에 대고 바람, p는 두 입술로 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q117" s="9" t="inlineStr">
+        <is>
+          <t>food /fuːd/ | pool /puːl/ | fee /fiː/ | pea /piː/</t>
+        </is>
+      </c>
+      <c r="R117" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S117" s="9" t="inlineStr"/>
+      <c r="T117" s="9" t="inlineStr"/>
+      <c r="U117" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V117" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W117" s="9" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="X117" s="9" t="inlineStr">
+        <is>
+          <t>급여, 봉급</t>
+        </is>
+      </c>
+      <c r="Y117" s="9" t="inlineStr">
+        <is>
+          <t>로마 병사는 소금(sal)으로 급여를 받았음. salt와 같은 어근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-02
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y117"/>
+  <dimension ref="A1:Y118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14223,6 +14223,123 @@
         </is>
       </c>
     </row>
+    <row r="118" ht="60" customHeight="1">
+      <c r="A118" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B118" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C118" s="9" t="inlineStr">
+        <is>
+          <t>비교급·최상급</t>
+        </is>
+      </c>
+      <c r="D118" s="9" t="inlineStr">
+        <is>
+          <t>Comparative and Superlative Adjectives</t>
+        </is>
+      </c>
+      <c r="E118" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F118" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G118" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H118" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I118" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Snow Queen</t>
+        </is>
+      </c>
+      <c r="J118" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K118" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L118" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M118" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N118" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O118" s="9" t="inlineStr">
+        <is>
+          <t>v vs b 구분</t>
+        </is>
+      </c>
+      <c r="P118" s="9" t="inlineStr">
+        <is>
+          <t>v는 윗니를 아랫입술에 대고 진동, b는 두 입술로 막아 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q118" s="9" t="inlineStr">
+        <is>
+          <t>very /véri/ | berry /béri/ | vest /vest/ | best /best/</t>
+        </is>
+      </c>
+      <c r="R118" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S118" s="9" t="inlineStr"/>
+      <c r="T118" s="9" t="inlineStr"/>
+      <c r="U118" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V118" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W118" s="9" t="inlineStr">
+        <is>
+          <t>muscle</t>
+        </is>
+      </c>
+      <c r="X118" s="9" t="inlineStr">
+        <is>
+          <t>근육</t>
+        </is>
+      </c>
+      <c r="Y118" s="9" t="inlineStr">
+        <is>
+          <t>팔을 구부릴 때 근육이 움직이는 모습이 쥐처럼 보인다 하여</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-03
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y118"/>
+  <dimension ref="A1:Y119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14340,6 +14340,123 @@
         </is>
       </c>
     </row>
+    <row r="119" ht="60" customHeight="1">
+      <c r="A119" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B119" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C119" s="9" t="inlineStr">
+        <is>
+          <t>장소 전치사</t>
+        </is>
+      </c>
+      <c r="D119" s="9" t="inlineStr">
+        <is>
+          <t>Prepositions of Place: at / in / on / by</t>
+        </is>
+      </c>
+      <c r="E119" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F119" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G119" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H119" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I119" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Snow Queen</t>
+        </is>
+      </c>
+      <c r="J119" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K119" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L119" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M119" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N119" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O119" s="9" t="inlineStr">
+        <is>
+          <t>th 유성음 /ð/</t>
+        </is>
+      </c>
+      <c r="P119" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 목소리 진동</t>
+        </is>
+      </c>
+      <c r="Q119" s="9" t="inlineStr">
+        <is>
+          <t>the /ðə/ | this /ðɪs/ | that /ðæt/ | mother /mʌðər/</t>
+        </is>
+      </c>
+      <c r="R119" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S119" s="9" t="inlineStr"/>
+      <c r="T119" s="9" t="inlineStr"/>
+      <c r="U119" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V119" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W119" s="9" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="X119" s="9" t="inlineStr">
+        <is>
+          <t>후보자</t>
+        </is>
+      </c>
+      <c r="Y119" s="9" t="inlineStr">
+        <is>
+          <t>로마 선거 출마자는 순결을 상징하는 흰 토가(candida)를 입었음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-04
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y119"/>
+  <dimension ref="A1:Y120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14457,6 +14457,123 @@
         </is>
       </c>
     </row>
+    <row r="120" ht="60" customHeight="1">
+      <c r="A120" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B120" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C120" s="9" t="inlineStr">
+        <is>
+          <t>단순과거 vs 과거진행</t>
+        </is>
+      </c>
+      <c r="D120" s="9" t="inlineStr">
+        <is>
+          <t>Past Simple vs Past Continuous</t>
+        </is>
+      </c>
+      <c r="E120" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F120" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G120" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H120" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I120" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Snow Queen</t>
+        </is>
+      </c>
+      <c r="J120" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K120" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L120" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M120" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N120" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O120" s="9" t="inlineStr">
+        <is>
+          <t>th 무성음 /θ/</t>
+        </is>
+      </c>
+      <c r="P120" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 바람만 내보냄</t>
+        </is>
+      </c>
+      <c r="Q120" s="9" t="inlineStr">
+        <is>
+          <t>think /θɪŋk/ | three /θriː/ | health /helθ/ | month /mʌnθ/</t>
+        </is>
+      </c>
+      <c r="R120" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S120" s="9" t="inlineStr"/>
+      <c r="T120" s="9" t="inlineStr"/>
+      <c r="U120" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V120" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W120" s="9" t="inlineStr">
+        <is>
+          <t>disaster</t>
+        </is>
+      </c>
+      <c r="X120" s="9" t="inlineStr">
+        <is>
+          <t>재앙, 참사</t>
+        </is>
+      </c>
+      <c r="Y120" s="9" t="inlineStr">
+        <is>
+          <t>별의 위치가 나쁘면 재앙이 온다는 점성술 믿음에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-06
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y120"/>
+  <dimension ref="A1:Y121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14574,6 +14574,123 @@
         </is>
       </c>
     </row>
+    <row r="121" ht="60" customHeight="1">
+      <c r="A121" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B121" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C121" s="9" t="inlineStr">
+        <is>
+          <t>명사절과 간접의문문</t>
+        </is>
+      </c>
+      <c r="D121" s="9" t="inlineStr">
+        <is>
+          <t>Noun Clauses and Embedded Questions</t>
+        </is>
+      </c>
+      <c r="E121" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F121" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G121" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H121" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I121" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Snow Queen</t>
+        </is>
+      </c>
+      <c r="J121" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K121" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L121" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M121" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N121" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O121" s="9" t="inlineStr">
+        <is>
+          <t>짧은 모음 vs 긴 모음</t>
+        </is>
+      </c>
+      <c r="P121" s="9" t="inlineStr">
+        <is>
+          <t>ship /ɪ/ vs sheep /iː/ — 입 모양과 길이 모두 다름</t>
+        </is>
+      </c>
+      <c r="Q121" s="9" t="inlineStr">
+        <is>
+          <t>ship /ʃɪp/ | sheep /ʃiːp/ | hit /hɪt/ | heat /hiːt/</t>
+        </is>
+      </c>
+      <c r="R121" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S121" s="9" t="inlineStr"/>
+      <c r="T121" s="9" t="inlineStr"/>
+      <c r="U121" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V121" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W121" s="9" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="X121" s="9" t="inlineStr">
+        <is>
+          <t>회사, 동료</t>
+        </is>
+      </c>
+      <c r="Y121" s="9" t="inlineStr">
+        <is>
+          <t>같이 빵을 나눠 먹는 동료에서 유래. companion(동료)과 동근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-07
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y122"/>
+  <dimension ref="A1:Y123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14808,6 +14808,123 @@
         </is>
       </c>
     </row>
+    <row r="123" ht="60" customHeight="1">
+      <c r="A123" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B123" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C123" s="9" t="inlineStr">
+        <is>
+          <t>능력·공손 조동사</t>
+        </is>
+      </c>
+      <c r="D123" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: can / could — 능력과 공손</t>
+        </is>
+      </c>
+      <c r="E123" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F123" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G123" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H123" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I123" s="9" t="inlineStr">
+        <is>
+          <t>discreet</t>
+        </is>
+      </c>
+      <c r="J123" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K123" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L123" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M123" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N123" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O123" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 명사</t>
+        </is>
+      </c>
+      <c r="P123" s="9" t="inlineStr">
+        <is>
+          <t>명사는 보통 첫 음절 강세 — REcord, PROtest, PERmit</t>
+        </is>
+      </c>
+      <c r="Q123" s="9" t="inlineStr">
+        <is>
+          <t>REcord | PROtest | PERmit | CONtent</t>
+        </is>
+      </c>
+      <c r="R123" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S123" s="9" t="inlineStr"/>
+      <c r="T123" s="9" t="inlineStr"/>
+      <c r="U123" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V123" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W123" s="9" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="X123" s="9" t="inlineStr">
+        <is>
+          <t>마감 기한</t>
+        </is>
+      </c>
+      <c r="Y123" s="9" t="inlineStr">
+        <is>
+          <t>남북전쟁 포로수용소에서 그 선을 넘으면 사살한다는 경계선에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-08
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y123"/>
+  <dimension ref="A1:Y124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14925,6 +14925,123 @@
         </is>
       </c>
     </row>
+    <row r="124" ht="60" customHeight="1">
+      <c r="A124" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B124" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C124" s="9" t="inlineStr">
+        <is>
+          <t>실현 가능한 조건문</t>
+        </is>
+      </c>
+      <c r="D124" s="9" t="inlineStr">
+        <is>
+          <t>First Conditional</t>
+        </is>
+      </c>
+      <c r="E124" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F124" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G124" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H124" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I124" s="9" t="inlineStr">
+        <is>
+          <t>etiquette</t>
+        </is>
+      </c>
+      <c r="J124" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K124" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L124" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M124" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N124" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O124" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 동사</t>
+        </is>
+      </c>
+      <c r="P124" s="9" t="inlineStr">
+        <is>
+          <t>동사는 보통 두 번째 음절 강세 — reCORD, proTEST, perMIT</t>
+        </is>
+      </c>
+      <c r="Q124" s="9" t="inlineStr">
+        <is>
+          <t>reCORD | proTEST | perMIT | conTENT</t>
+        </is>
+      </c>
+      <c r="R124" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S124" s="9" t="inlineStr"/>
+      <c r="T124" s="9" t="inlineStr"/>
+      <c r="U124" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V124" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W124" s="9" t="inlineStr">
+        <is>
+          <t>bankrupt</t>
+        </is>
+      </c>
+      <c r="X124" s="9" t="inlineStr">
+        <is>
+          <t>파산한</t>
+        </is>
+      </c>
+      <c r="Y124" s="9" t="inlineStr">
+        <is>
+          <t>중세 환전상이 파산하면 거래 탁자(banca)를 부수는 관습에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-09
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y124"/>
+  <dimension ref="A1:Y125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15042,6 +15042,123 @@
         </is>
       </c>
     </row>
+    <row r="125" ht="60" customHeight="1">
+      <c r="A125" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B125" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C125" s="9" t="inlineStr">
+        <is>
+          <t>수동태</t>
+        </is>
+      </c>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>Passive Voice</t>
+        </is>
+      </c>
+      <c r="E125" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F125" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G125" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H125" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I125" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Cinderella</t>
+        </is>
+      </c>
+      <c r="J125" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K125" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L125" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M125" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N125" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O125" s="9" t="inlineStr">
+        <is>
+          <t>-ed 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P125" s="9" t="inlineStr">
+        <is>
+          <t>/t/: 무성음 뒤 | /d/: 유성음 뒤 | /ɪd/: t·d로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q125" s="9" t="inlineStr">
+        <is>
+          <t>worked /wɜːrkt/ | called /kɔːld/ | wanted /wɒntɪd/ | needed /niːdɪd/</t>
+        </is>
+      </c>
+      <c r="R125" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S125" s="9" t="inlineStr"/>
+      <c r="T125" s="9" t="inlineStr"/>
+      <c r="U125" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V125" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W125" s="9" t="inlineStr">
+        <is>
+          <t>quiz</t>
+        </is>
+      </c>
+      <c r="X125" s="9" t="inlineStr">
+        <is>
+          <t>퀴즈, 시험</t>
+        </is>
+      </c>
+      <c r="Y125" s="9" t="inlineStr">
+        <is>
+          <t>더블린 극장주 Daly가 무의미한 단어를 낙서하면 하루 만에 유행어로 만든 일화에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-10
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y125"/>
+  <dimension ref="A1:Y126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15159,6 +15159,123 @@
         </is>
       </c>
     </row>
+    <row r="126" ht="60" customHeight="1">
+      <c r="A126" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B126" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C126" s="9" t="inlineStr">
+        <is>
+          <t>관사</t>
+        </is>
+      </c>
+      <c r="D126" s="9" t="inlineStr">
+        <is>
+          <t>Articles: a / an / the</t>
+        </is>
+      </c>
+      <c r="E126" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F126" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G126" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H126" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I126" s="9" t="inlineStr">
+        <is>
+          <t>Luddite</t>
+        </is>
+      </c>
+      <c r="J126" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K126" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L126" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M126" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N126" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O126" s="9" t="inlineStr">
+        <is>
+          <t>-s/-es 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P126" s="9" t="inlineStr">
+        <is>
+          <t>/ s/: 무성음 뒤 | /z/: 유성음 뒤 | /ɪz/: s·z·ch·sh로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q126" s="9" t="inlineStr">
+        <is>
+          <t>books /bʊks/ | dogs /dɒgz/ | watches /wɒtʃɪz/ | buses /bʌsɪz/</t>
+        </is>
+      </c>
+      <c r="R126" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S126" s="9" t="inlineStr"/>
+      <c r="T126" s="9" t="inlineStr"/>
+      <c r="U126" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V126" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W126" s="9" t="inlineStr">
+        <is>
+          <t>panic</t>
+        </is>
+      </c>
+      <c r="X126" s="9" t="inlineStr">
+        <is>
+          <t>공황, 극도의 공포</t>
+        </is>
+      </c>
+      <c r="Y126" s="9" t="inlineStr">
+        <is>
+          <t>목신 판(Pan)이 갑자기 나타나 공포를 일으킨다는 신화에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-11
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y126"/>
+  <dimension ref="A1:Y127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15276,6 +15276,123 @@
         </is>
       </c>
     </row>
+    <row r="127" ht="60" customHeight="1">
+      <c r="A127" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B127" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C127" s="9" t="inlineStr">
+        <is>
+          <t>강조 도치</t>
+        </is>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>Inversion for Emphasis</t>
+        </is>
+      </c>
+      <c r="E127" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F127" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G127" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H127" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I127" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Cinderella</t>
+        </is>
+      </c>
+      <c r="J127" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K127" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L127" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M127" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N127" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O127" s="9" t="inlineStr">
+        <is>
+          <t>연음 (Linking)</t>
+        </is>
+      </c>
+      <c r="P127" s="9" t="inlineStr">
+        <is>
+          <t>자음으로 끝나는 단어 + 모음으로 시작하는 단어는 이어서 발음</t>
+        </is>
+      </c>
+      <c r="Q127" s="9" t="inlineStr">
+        <is>
+          <t>pick it up → pi-ki-tup | turn it on → tur-ni-ton | look at it → loo-ka-tit</t>
+        </is>
+      </c>
+      <c r="R127" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S127" s="9" t="inlineStr"/>
+      <c r="T127" s="9" t="inlineStr"/>
+      <c r="U127" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V127" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W127" s="9" t="inlineStr">
+        <is>
+          <t>strategy</t>
+        </is>
+      </c>
+      <c r="X127" s="9" t="inlineStr">
+        <is>
+          <t>전략</t>
+        </is>
+      </c>
+      <c r="Y127" s="9" t="inlineStr">
+        <is>
+          <t>stratos(군대) + agein(이끌다) → 장군의 기술</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-13
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y127"/>
+  <dimension ref="A1:Y128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15393,6 +15393,123 @@
         </is>
       </c>
     </row>
+    <row r="128" ht="60" customHeight="1">
+      <c r="A128" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B128" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C128" s="9" t="inlineStr">
+        <is>
+          <t>과거완료</t>
+        </is>
+      </c>
+      <c r="D128" s="9" t="inlineStr">
+        <is>
+          <t>Past Perfect Tense</t>
+        </is>
+      </c>
+      <c r="E128" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F128" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G128" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H128" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I128" s="9" t="inlineStr">
+        <is>
+          <t>nexus</t>
+        </is>
+      </c>
+      <c r="J128" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K128" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L128" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M128" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N128" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O128" s="9" t="inlineStr">
+        <is>
+          <t>약화 (Reduction)</t>
+        </is>
+      </c>
+      <c r="P128" s="9" t="inlineStr">
+        <is>
+          <t>기능어(of·to·for·and·at)는 빠르게 약화 — /ə/ 로 줄어듦</t>
+        </is>
+      </c>
+      <c r="Q128" s="9" t="inlineStr">
+        <is>
+          <t>cup of tea → cupə tea | a lot of → ə lɒtə | want to → wanna</t>
+        </is>
+      </c>
+      <c r="R128" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S128" s="9" t="inlineStr"/>
+      <c r="T128" s="9" t="inlineStr"/>
+      <c r="U128" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V128" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W128" s="9" t="inlineStr">
+        <is>
+          <t>focus</t>
+        </is>
+      </c>
+      <c r="X128" s="9" t="inlineStr">
+        <is>
+          <t>초점, 집중</t>
+        </is>
+      </c>
+      <c r="Y128" s="9" t="inlineStr">
+        <is>
+          <t>로마 가정의 화덕이 집의 중심이었던 데서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-14
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y129"/>
+  <dimension ref="A1:Y130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15627,6 +15627,123 @@
         </is>
       </c>
     </row>
+    <row r="130" ht="60" customHeight="1">
+      <c r="A130" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B130" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C130" s="9" t="inlineStr">
+        <is>
+          <t>가정법 과거</t>
+        </is>
+      </c>
+      <c r="D130" s="9" t="inlineStr">
+        <is>
+          <t>Second Conditional</t>
+        </is>
+      </c>
+      <c r="E130" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F130" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G130" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H130" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I130" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Cinderella</t>
+        </is>
+      </c>
+      <c r="J130" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K130" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L130" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M130" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N130" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O130" s="9" t="inlineStr">
+        <is>
+          <t>억양: 의문문</t>
+        </is>
+      </c>
+      <c r="P130" s="9" t="inlineStr">
+        <is>
+          <t>Yes/No 질문은 끝이 올라가고 ↗, Wh- 질문은 끝이 내려감 ↘</t>
+        </is>
+      </c>
+      <c r="Q130" s="9" t="inlineStr">
+        <is>
+          <t>Are you READY? ↗ | Where are you GOING? ↘ | Did you SEE it? ↗</t>
+        </is>
+      </c>
+      <c r="R130" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S130" s="9" t="inlineStr"/>
+      <c r="T130" s="9" t="inlineStr"/>
+      <c r="U130" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V130" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W130" s="9" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="X130" s="9" t="inlineStr">
+        <is>
+          <t>위험, 위험을 감수하다</t>
+        </is>
+      </c>
+      <c r="Y130" s="9" t="inlineStr">
+        <is>
+          <t>항해 중 암초 근처를 항행하는 위험에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-15
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y130"/>
+  <dimension ref="A1:Y131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15744,6 +15744,123 @@
         </is>
       </c>
     </row>
+    <row r="131" ht="60" customHeight="1">
+      <c r="A131" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B131" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C131" s="9" t="inlineStr">
+        <is>
+          <t>간접화법</t>
+        </is>
+      </c>
+      <c r="D131" s="9" t="inlineStr">
+        <is>
+          <t>Reported Speech</t>
+        </is>
+      </c>
+      <c r="E131" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F131" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G131" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H131" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I131" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Cinderella</t>
+        </is>
+      </c>
+      <c r="J131" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K131" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L131" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M131" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N131" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O131" s="9" t="inlineStr">
+        <is>
+          <t>r vs l 구분</t>
+        </is>
+      </c>
+      <c r="P131" s="9" t="inlineStr">
+        <is>
+          <t>r은 혀를 말아 입천장에 닿지 않게, l은 혀끝을 윗잇몸에 확실히 댐</t>
+        </is>
+      </c>
+      <c r="Q131" s="9" t="inlineStr">
+        <is>
+          <t>really /ríːli/ | rally /réli/ | river /rívər/ | liver /lívər/</t>
+        </is>
+      </c>
+      <c r="R131" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S131" s="9" t="inlineStr"/>
+      <c r="T131" s="9" t="inlineStr"/>
+      <c r="U131" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V131" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W131" s="9" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
+      <c r="X131" s="9" t="inlineStr">
+        <is>
+          <t>예산</t>
+        </is>
+      </c>
+      <c r="Y131" s="9" t="inlineStr">
+        <is>
+          <t>재무장관이 예산서를 담은 가죽 가방(bougette)을 들고 의회에 출석한 데서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-16
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y131"/>
+  <dimension ref="A1:Y132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15861,6 +15861,123 @@
         </is>
       </c>
     </row>
+    <row r="132" ht="60" customHeight="1">
+      <c r="A132" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B132" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C132" s="9" t="inlineStr">
+        <is>
+          <t>동명사 vs 부정사</t>
+        </is>
+      </c>
+      <c r="D132" s="9" t="inlineStr">
+        <is>
+          <t>Gerunds vs Infinitives</t>
+        </is>
+      </c>
+      <c r="E132" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F132" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G132" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H132" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I132" s="9" t="inlineStr">
+        <is>
+          <t>zenith</t>
+        </is>
+      </c>
+      <c r="J132" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K132" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L132" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M132" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N132" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O132" s="9" t="inlineStr">
+        <is>
+          <t>f vs p 구분</t>
+        </is>
+      </c>
+      <c r="P132" s="9" t="inlineStr">
+        <is>
+          <t>f는 윗니를 아랫입술에 대고 바람, p는 두 입술로 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q132" s="9" t="inlineStr">
+        <is>
+          <t>food /fuːd/ | pool /puːl/ | fee /fiː/ | pea /piː/</t>
+        </is>
+      </c>
+      <c r="R132" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S132" s="9" t="inlineStr"/>
+      <c r="T132" s="9" t="inlineStr"/>
+      <c r="U132" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V132" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W132" s="9" t="inlineStr">
+        <is>
+          <t>magazine</t>
+        </is>
+      </c>
+      <c r="X132" s="9" t="inlineStr">
+        <is>
+          <t>잡지, 탄창</t>
+        </is>
+      </c>
+      <c r="Y132" s="9" t="inlineStr">
+        <is>
+          <t>지식·정보를 저장해 두는 '창고'라는 의미로 출판물에 사용됨</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-17
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y132"/>
+  <dimension ref="A1:Y133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15978,6 +15978,123 @@
         </is>
       </c>
     </row>
+    <row r="133" ht="60" customHeight="1">
+      <c r="A133" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B133" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C133" s="9" t="inlineStr">
+        <is>
+          <t>가정법 현재 (요구·제안 구문)</t>
+        </is>
+      </c>
+      <c r="D133" s="9" t="inlineStr">
+        <is>
+          <t>Subjunctive Mood</t>
+        </is>
+      </c>
+      <c r="E133" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F133" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G133" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H133" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I133" s="9" t="inlineStr">
+        <is>
+          <t>syncretic</t>
+        </is>
+      </c>
+      <c r="J133" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K133" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L133" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M133" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N133" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O133" s="9" t="inlineStr">
+        <is>
+          <t>v vs b 구분</t>
+        </is>
+      </c>
+      <c r="P133" s="9" t="inlineStr">
+        <is>
+          <t>v는 윗니를 아랫입술에 대고 진동, b는 두 입술로 막아 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q133" s="9" t="inlineStr">
+        <is>
+          <t>very /véri/ | berry /béri/ | vest /vest/ | best /best/</t>
+        </is>
+      </c>
+      <c r="R133" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S133" s="9" t="inlineStr"/>
+      <c r="T133" s="9" t="inlineStr"/>
+      <c r="U133" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V133" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W133" s="9" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="X133" s="9" t="inlineStr">
+        <is>
+          <t>후보자</t>
+        </is>
+      </c>
+      <c r="Y133" s="9" t="inlineStr">
+        <is>
+          <t>로마 선거 출마자는 순결을 상징하는 흰 토가를 입었음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-18
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y133"/>
+  <dimension ref="A1:Y134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16095,6 +16095,123 @@
         </is>
       </c>
     </row>
+    <row r="134" ht="60" customHeight="1">
+      <c r="A134" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B134" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>미래 표현 3가지</t>
+        </is>
+      </c>
+      <c r="D134" s="9" t="inlineStr">
+        <is>
+          <t>Future Tenses: will / going to / present continuous</t>
+        </is>
+      </c>
+      <c r="E134" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F134" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G134" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H134" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I134" s="9" t="inlineStr">
+        <is>
+          <t>bon vivant</t>
+        </is>
+      </c>
+      <c r="J134" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K134" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L134" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M134" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N134" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O134" s="9" t="inlineStr">
+        <is>
+          <t>th 유성음 /ð/</t>
+        </is>
+      </c>
+      <c r="P134" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 목소리 진동</t>
+        </is>
+      </c>
+      <c r="Q134" s="9" t="inlineStr">
+        <is>
+          <t>the /ðə/ | this /ðɪs/ | that /ðæt/ | mother /mʌðər/</t>
+        </is>
+      </c>
+      <c r="R134" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S134" s="9" t="inlineStr"/>
+      <c r="T134" s="9" t="inlineStr"/>
+      <c r="U134" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V134" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W134" s="9" t="inlineStr">
+        <is>
+          <t>serendipity</t>
+        </is>
+      </c>
+      <c r="X134" s="9" t="inlineStr">
+        <is>
+          <t>뜻밖의 행운</t>
+        </is>
+      </c>
+      <c r="Y134" s="9" t="inlineStr">
+        <is>
+          <t>세 왕자가 우연히 훌륭한 발견을 하는 동화에서 Horace Walpole이 만든 단어</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-19
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y134"/>
+  <dimension ref="A1:Y135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16212,6 +16212,123 @@
         </is>
       </c>
     </row>
+    <row r="135" ht="60" customHeight="1">
+      <c r="A135" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B135" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C135" s="9" t="inlineStr">
+        <is>
+          <t>의무·필요 조동사</t>
+        </is>
+      </c>
+      <c r="D135" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: must / have to / need to</t>
+        </is>
+      </c>
+      <c r="E135" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F135" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G135" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H135" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I135" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Adventures of Huckleberry Finn</t>
+        </is>
+      </c>
+      <c r="J135" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K135" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L135" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M135" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N135" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O135" s="9" t="inlineStr">
+        <is>
+          <t>th 무성음 /θ/</t>
+        </is>
+      </c>
+      <c r="P135" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 바람만 내보냄</t>
+        </is>
+      </c>
+      <c r="Q135" s="9" t="inlineStr">
+        <is>
+          <t>think /θɪŋk/ | three /θriː/ | health /helθ/ | month /mʌnθ/</t>
+        </is>
+      </c>
+      <c r="R135" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S135" s="9" t="inlineStr"/>
+      <c r="T135" s="9" t="inlineStr"/>
+      <c r="U135" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V135" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W135" s="9" t="inlineStr">
+        <is>
+          <t>berserk</t>
+        </is>
+      </c>
+      <c r="X135" s="9" t="inlineStr">
+        <is>
+          <t>극도로 흥분한, 폭주하는</t>
+        </is>
+      </c>
+      <c r="Y135" s="9" t="inlineStr">
+        <is>
+          <t>전투에서 곰 가죽을 입고 광분하던 바이킹 전사에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-20
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y135"/>
+  <dimension ref="A1:Y136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16329,6 +16329,123 @@
         </is>
       </c>
     </row>
+    <row r="136" ht="60" customHeight="1">
+      <c r="A136" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B136" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C136" s="9" t="inlineStr">
+        <is>
+          <t>가정법 과거완료·혼합</t>
+        </is>
+      </c>
+      <c r="D136" s="9" t="inlineStr">
+        <is>
+          <t>Third Conditional &amp; Mixed Conditionals</t>
+        </is>
+      </c>
+      <c r="E136" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F136" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G136" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H136" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I136" s="9" t="inlineStr">
+        <is>
+          <t>compunction</t>
+        </is>
+      </c>
+      <c r="J136" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K136" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L136" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M136" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N136" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O136" s="9" t="inlineStr">
+        <is>
+          <t>짧은 모음 vs 긴 모음</t>
+        </is>
+      </c>
+      <c r="P136" s="9" t="inlineStr">
+        <is>
+          <t>ship /ɪ/ vs sheep /iː/ — 입 모양과 길이 모두 다름</t>
+        </is>
+      </c>
+      <c r="Q136" s="9" t="inlineStr">
+        <is>
+          <t>ship /ʃɪp/ | sheep /ʃiːp/ | hit /hɪt/ | heat /hiːt/</t>
+        </is>
+      </c>
+      <c r="R136" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S136" s="9" t="inlineStr"/>
+      <c r="T136" s="9" t="inlineStr"/>
+      <c r="U136" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V136" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W136" s="9" t="inlineStr">
+        <is>
+          <t>boycott</t>
+        </is>
+      </c>
+      <c r="X136" s="9" t="inlineStr">
+        <is>
+          <t>불매운동, 거부하다</t>
+        </is>
+      </c>
+      <c r="Y136" s="9" t="inlineStr">
+        <is>
+          <t>1880년 소작인들이 Boycott을 집단 거부한 사건에서 단어화</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-21
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y136"/>
+  <dimension ref="A1:Y137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16446,6 +16446,123 @@
         </is>
       </c>
     </row>
+    <row r="137" ht="60" customHeight="1">
+      <c r="A137" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B137" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C137" s="9" t="inlineStr">
+        <is>
+          <t>관계절</t>
+        </is>
+      </c>
+      <c r="D137" s="9" t="inlineStr">
+        <is>
+          <t>Relative Clauses: defining vs non-defining</t>
+        </is>
+      </c>
+      <c r="E137" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F137" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G137" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H137" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I137" s="9" t="inlineStr">
+        <is>
+          <t>jilt</t>
+        </is>
+      </c>
+      <c r="J137" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K137" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L137" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M137" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N137" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O137" s="9" t="inlineStr">
+        <is>
+          <t>어말 자음 탈락 방지</t>
+        </is>
+      </c>
+      <c r="P137" s="9" t="inlineStr">
+        <is>
+          <t>한국어는 받침 뒤 모음을 붙이는 경향 — 마지막 자음만 닫고 끝내기</t>
+        </is>
+      </c>
+      <c r="Q137" s="9" t="inlineStr">
+        <is>
+          <t>fact /fækt/ | next /nekst/ | helped /helpt/ | asked /æskt/</t>
+        </is>
+      </c>
+      <c r="R137" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S137" s="9" t="inlineStr"/>
+      <c r="T137" s="9" t="inlineStr"/>
+      <c r="U137" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V137" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W137" s="9" t="inlineStr">
+        <is>
+          <t>mentor</t>
+        </is>
+      </c>
+      <c r="X137" s="9" t="inlineStr">
+        <is>
+          <t>멘토, 스승</t>
+        </is>
+      </c>
+      <c r="Y137" s="9" t="inlineStr">
+        <is>
+          <t>오디세우스가 트로이 전쟁 중 아들 텔레마코스 교육을 맡긴 현자의 이름에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-22
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y137"/>
+  <dimension ref="A1:Y138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16563,6 +16563,123 @@
         </is>
       </c>
     </row>
+    <row r="138" ht="60" customHeight="1">
+      <c r="A138" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B138" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C138" s="9" t="inlineStr">
+        <is>
+          <t>시간 전치사</t>
+        </is>
+      </c>
+      <c r="D138" s="9" t="inlineStr">
+        <is>
+          <t>Prepositions of Time: at / in / on / by</t>
+        </is>
+      </c>
+      <c r="E138" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F138" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G138" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H138" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I138" s="9" t="inlineStr">
+        <is>
+          <t>vocation</t>
+        </is>
+      </c>
+      <c r="J138" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K138" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L138" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M138" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N138" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O138" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 명사</t>
+        </is>
+      </c>
+      <c r="P138" s="9" t="inlineStr">
+        <is>
+          <t>명사는 보통 첫 음절 강세 — REcord, PROtest, PERmit</t>
+        </is>
+      </c>
+      <c r="Q138" s="9" t="inlineStr">
+        <is>
+          <t>REcord | PROtest | PERmit | CONtent</t>
+        </is>
+      </c>
+      <c r="R138" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S138" s="9" t="inlineStr"/>
+      <c r="T138" s="9" t="inlineStr"/>
+      <c r="U138" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V138" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W138" s="9" t="inlineStr">
+        <is>
+          <t>rival</t>
+        </is>
+      </c>
+      <c r="X138" s="9" t="inlineStr">
+        <is>
+          <t>경쟁자</t>
+        </is>
+      </c>
+      <c r="Y138" s="9" t="inlineStr">
+        <is>
+          <t>같은 강(rivus) 물을 사용하는 이웃 사이의 경쟁 관계에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-23
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y138"/>
+  <dimension ref="A1:Y139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16680,6 +16680,123 @@
         </is>
       </c>
     </row>
+    <row r="139" ht="60" customHeight="1">
+      <c r="A139" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B139" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C139" s="9" t="inlineStr">
+        <is>
+          <t>생략과 대용</t>
+        </is>
+      </c>
+      <c r="D139" s="9" t="inlineStr">
+        <is>
+          <t>Ellipsis and Substitution</t>
+        </is>
+      </c>
+      <c r="E139" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F139" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G139" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H139" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I139" s="9" t="inlineStr">
+        <is>
+          <t>asunder</t>
+        </is>
+      </c>
+      <c r="J139" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K139" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L139" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M139" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N139" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O139" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 동사</t>
+        </is>
+      </c>
+      <c r="P139" s="9" t="inlineStr">
+        <is>
+          <t>동사는 보통 두 번째 음절 강세 — reCORD, proTEST, perMIT</t>
+        </is>
+      </c>
+      <c r="Q139" s="9" t="inlineStr">
+        <is>
+          <t>reCORD | proTEST | perMIT | conTENT</t>
+        </is>
+      </c>
+      <c r="R139" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S139" s="9" t="inlineStr"/>
+      <c r="T139" s="9" t="inlineStr"/>
+      <c r="U139" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V139" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W139" s="9" t="inlineStr">
+        <is>
+          <t>travel</t>
+        </is>
+      </c>
+      <c r="X139" s="9" t="inlineStr">
+        <is>
+          <t>여행하다</t>
+        </is>
+      </c>
+      <c r="Y139" s="9" t="inlineStr">
+        <is>
+          <t>중세 여행이 고문(tripalium)처럼 고달팠던 데서 travail(고통)과 동근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-24
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y139"/>
+  <dimension ref="A1:Y140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16797,6 +16797,123 @@
         </is>
       </c>
     </row>
+    <row r="140" ht="60" customHeight="1">
+      <c r="A140" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B140" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C140" s="9" t="inlineStr">
+        <is>
+          <t>단순현재 vs 현재진행</t>
+        </is>
+      </c>
+      <c r="D140" s="9" t="inlineStr">
+        <is>
+          <t>Present Simple vs Present Continuous</t>
+        </is>
+      </c>
+      <c r="E140" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F140" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G140" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H140" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I140" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Adventures of Huckleberry Finn</t>
+        </is>
+      </c>
+      <c r="J140" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K140" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L140" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M140" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N140" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O140" s="9" t="inlineStr">
+        <is>
+          <t>-ed 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P140" s="9" t="inlineStr">
+        <is>
+          <t>/t/: 무성음 뒤 | /d/: 유성음 뒤 | /ɪd/: t·d로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q140" s="9" t="inlineStr">
+        <is>
+          <t>worked /wɜːrkt/ | called /kɔːld/ | wanted /wɒntɪd/ | needed /niːdɪd/</t>
+        </is>
+      </c>
+      <c r="R140" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S140" s="9" t="inlineStr"/>
+      <c r="T140" s="9" t="inlineStr"/>
+      <c r="U140" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V140" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W140" s="9" t="inlineStr">
+        <is>
+          <t>enthusiasm</t>
+        </is>
+      </c>
+      <c r="X140" s="9" t="inlineStr">
+        <is>
+          <t>열정, 열의</t>
+        </is>
+      </c>
+      <c r="Y140" s="9" t="inlineStr">
+        <is>
+          <t>en(안에) + theos(신) → 신에게 감화받은 열정 상태</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-25
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y140"/>
+  <dimension ref="A1:Y141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16914,6 +16914,123 @@
         </is>
       </c>
     </row>
+    <row r="141" ht="60" customHeight="1">
+      <c r="A141" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B141" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C141" s="9" t="inlineStr">
+        <is>
+          <t>구동사 (비즈니스)</t>
+        </is>
+      </c>
+      <c r="D141" s="9" t="inlineStr">
+        <is>
+          <t>Phrasal Verbs – Business Context</t>
+        </is>
+      </c>
+      <c r="E141" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F141" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G141" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H141" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I141" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Adventures of Huckleberry Finn</t>
+        </is>
+      </c>
+      <c r="J141" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K141" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L141" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M141" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N141" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O141" s="9" t="inlineStr">
+        <is>
+          <t>-s/-es 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P141" s="9" t="inlineStr">
+        <is>
+          <t>/ s/: 무성음 뒤 | /z/: 유성음 뒤 | /ɪz/: s·z·ch·sh로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q141" s="9" t="inlineStr">
+        <is>
+          <t>books /bʊks/ | dogs /dɒgz/ | watches /wɒtʃɪz/ | buses /bʌsɪz/</t>
+        </is>
+      </c>
+      <c r="R141" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S141" s="9" t="inlineStr"/>
+      <c r="T141" s="9" t="inlineStr"/>
+      <c r="U141" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V141" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W141" s="9" t="inlineStr">
+        <is>
+          <t>lucid</t>
+        </is>
+      </c>
+      <c r="X141" s="9" t="inlineStr">
+        <is>
+          <t>명확한, 이해하기 쉬운</t>
+        </is>
+      </c>
+      <c r="Y141" s="9" t="inlineStr">
+        <is>
+          <t>lux(빛)과 동근 → 명확하고 투명한 사고</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-26
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y141"/>
+  <dimension ref="A1:Y142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17031,6 +17031,123 @@
         </is>
       </c>
     </row>
+    <row r="142" ht="60" customHeight="1">
+      <c r="A142" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B142" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C142" s="9" t="inlineStr">
+        <is>
+          <t>비교급·최상급</t>
+        </is>
+      </c>
+      <c r="D142" s="9" t="inlineStr">
+        <is>
+          <t>Comparative and Superlative Adjectives</t>
+        </is>
+      </c>
+      <c r="E142" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F142" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G142" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H142" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I142" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Adventures of Huckleberry Finn</t>
+        </is>
+      </c>
+      <c r="J142" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K142" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L142" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M142" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N142" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O142" s="9" t="inlineStr">
+        <is>
+          <t>연음 (Linking)</t>
+        </is>
+      </c>
+      <c r="P142" s="9" t="inlineStr">
+        <is>
+          <t>자음으로 끝나는 단어 + 모음으로 시작하는 단어는 이어서 발음</t>
+        </is>
+      </c>
+      <c r="Q142" s="9" t="inlineStr">
+        <is>
+          <t>pick it up → pi-ki-tup | turn it on → tur-ni-ton | look at it → loo-ka-tit</t>
+        </is>
+      </c>
+      <c r="R142" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S142" s="9" t="inlineStr"/>
+      <c r="T142" s="9" t="inlineStr"/>
+      <c r="U142" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V142" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W142" s="9" t="inlineStr">
+        <is>
+          <t>colleague</t>
+        </is>
+      </c>
+      <c r="X142" s="9" t="inlineStr">
+        <is>
+          <t>동료</t>
+        </is>
+      </c>
+      <c r="Y142" s="9" t="inlineStr">
+        <is>
+          <t>col(함께) + legare(선택하다/보내다) → 같이 선발된 동료</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-27
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y142"/>
+  <dimension ref="A1:Y143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17148,6 +17148,123 @@
         </is>
       </c>
     </row>
+    <row r="143" ht="60" customHeight="1">
+      <c r="A143" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B143" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C143" s="9" t="inlineStr">
+        <is>
+          <t>장소 전치사</t>
+        </is>
+      </c>
+      <c r="D143" s="9" t="inlineStr">
+        <is>
+          <t>Prepositions of Place: at / in / on / by</t>
+        </is>
+      </c>
+      <c r="E143" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F143" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G143" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H143" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I143" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Adventures of Huckleberry Finn</t>
+        </is>
+      </c>
+      <c r="J143" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K143" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L143" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M143" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N143" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O143" s="9" t="inlineStr">
+        <is>
+          <t>약화 (Reduction)</t>
+        </is>
+      </c>
+      <c r="P143" s="9" t="inlineStr">
+        <is>
+          <t>기능어(of·to·for·and·at)는 빠르게 약화 — /ə/ 로 줄어듦</t>
+        </is>
+      </c>
+      <c r="Q143" s="9" t="inlineStr">
+        <is>
+          <t>cup of tea → cupə tea | a lot of → ə lɒtə | want to → wanna</t>
+        </is>
+      </c>
+      <c r="R143" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S143" s="9" t="inlineStr"/>
+      <c r="T143" s="9" t="inlineStr"/>
+      <c r="U143" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V143" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W143" s="9" t="inlineStr">
+        <is>
+          <t>quarantine</t>
+        </is>
+      </c>
+      <c r="X143" s="9" t="inlineStr">
+        <is>
+          <t>격리, 검역</t>
+        </is>
+      </c>
+      <c r="Y143" s="9" t="inlineStr">
+        <is>
+          <t>14세기 흑사병 때 선박을 40일간 격리한 베네치아 방역 정책에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-28
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y143"/>
+  <dimension ref="A1:Y144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17265,6 +17265,123 @@
         </is>
       </c>
     </row>
+    <row r="144" ht="60" customHeight="1">
+      <c r="A144" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B144" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C144" s="9" t="inlineStr">
+        <is>
+          <t>단순과거 vs 과거진행</t>
+        </is>
+      </c>
+      <c r="D144" s="9" t="inlineStr">
+        <is>
+          <t>Past Simple vs Past Continuous</t>
+        </is>
+      </c>
+      <c r="E144" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F144" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G144" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H144" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I144" s="9" t="inlineStr">
+        <is>
+          <t>grotesque</t>
+        </is>
+      </c>
+      <c r="J144" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K144" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L144" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M144" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N144" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O144" s="9" t="inlineStr">
+        <is>
+          <t>문장 강세와 리듬</t>
+        </is>
+      </c>
+      <c r="P144" s="9" t="inlineStr">
+        <is>
+          <t>내용어(명사·동사·형용사)는 강하게, 기능어(관사·전치사)는 약하게</t>
+        </is>
+      </c>
+      <c r="Q144" s="9" t="inlineStr">
+        <is>
+          <t>I WANT to GO to the STORE | She's WORKING on a NEW project</t>
+        </is>
+      </c>
+      <c r="R144" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S144" s="9" t="inlineStr"/>
+      <c r="T144" s="9" t="inlineStr"/>
+      <c r="U144" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V144" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W144" s="9" t="inlineStr">
+        <is>
+          <t>clue</t>
+        </is>
+      </c>
+      <c r="X144" s="9" t="inlineStr">
+        <is>
+          <t>단서, 실마리</t>
+        </is>
+      </c>
+      <c r="Y144" s="9" t="inlineStr">
+        <is>
+          <t>그리스 신화에서 테세우스가 미로를 탈출할 때 아리아드네의 실(clew)에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-29
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y144"/>
+  <dimension ref="A1:Y145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17382,6 +17382,123 @@
         </is>
       </c>
     </row>
+    <row r="145" ht="60" customHeight="1">
+      <c r="A145" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B145" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C145" s="9" t="inlineStr">
+        <is>
+          <t>명사절과 간접의문문</t>
+        </is>
+      </c>
+      <c r="D145" s="9" t="inlineStr">
+        <is>
+          <t>Noun Clauses and Embedded Questions</t>
+        </is>
+      </c>
+      <c r="E145" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F145" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G145" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H145" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I145" s="9" t="inlineStr">
+        <is>
+          <t>shindig</t>
+        </is>
+      </c>
+      <c r="J145" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K145" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L145" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M145" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N145" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O145" s="9" t="inlineStr">
+        <is>
+          <t>억양: 의문문</t>
+        </is>
+      </c>
+      <c r="P145" s="9" t="inlineStr">
+        <is>
+          <t>Yes/No 질문은 끝이 올라가고 ↗, Wh- 질문은 끝이 내려감 ↘</t>
+        </is>
+      </c>
+      <c r="Q145" s="9" t="inlineStr">
+        <is>
+          <t>Are you READY? ↗ | Where are you GOING? ↘ | Did you SEE it? ↗</t>
+        </is>
+      </c>
+      <c r="R145" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S145" s="9" t="inlineStr"/>
+      <c r="T145" s="9" t="inlineStr"/>
+      <c r="U145" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V145" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W145" s="9" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="X145" s="9" t="inlineStr">
+        <is>
+          <t>급여</t>
+        </is>
+      </c>
+      <c r="Y145" s="9" t="inlineStr">
+        <is>
+          <t>로마 병사의 소금 급여에서. '소금값 못하는 사람'이라는 표현도 여기서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-10-30
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y145"/>
+  <dimension ref="A1:Y146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17499,6 +17499,123 @@
         </is>
       </c>
     </row>
+    <row r="146" ht="60" customHeight="1">
+      <c r="A146" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B146" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C146" s="9" t="inlineStr">
+        <is>
+          <t>현재완료 vs 단순과거</t>
+        </is>
+      </c>
+      <c r="D146" s="9" t="inlineStr">
+        <is>
+          <t>Present Perfect vs Simple Past</t>
+        </is>
+      </c>
+      <c r="E146" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F146" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G146" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H146" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I146" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Island of Dr Moreau</t>
+        </is>
+      </c>
+      <c r="J146" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a common English expression used in business settings. When someone says 'Let's take this offline,' they mean continuing a conversation privately, outside the current meeting.</t>
+        </is>
+      </c>
+      <c r="K146" s="9" t="inlineStr">
+        <is>
+          <t>offline — 회의 밖에서 (오프라인 X); take [something] offline — 나중에 따로 논의하다</t>
+        </is>
+      </c>
+      <c r="L146" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M146" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N146" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O146" s="9" t="inlineStr">
+        <is>
+          <t>r vs l 구분</t>
+        </is>
+      </c>
+      <c r="P146" s="9" t="inlineStr">
+        <is>
+          <t>r은 혀를 말아 입천장에 닿지 않게, l은 혀끝을 윗잇몸에 확실히 댐</t>
+        </is>
+      </c>
+      <c r="Q146" s="9" t="inlineStr">
+        <is>
+          <t>really /ríːli/ | rally /réli/ | river /rívər/ | liver /lívər/</t>
+        </is>
+      </c>
+      <c r="R146" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S146" s="9" t="inlineStr"/>
+      <c r="T146" s="9" t="inlineStr"/>
+      <c r="U146" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V146" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W146" s="9" t="inlineStr">
+        <is>
+          <t>sincere</t>
+        </is>
+      </c>
+      <c r="X146" s="9" t="inlineStr">
+        <is>
+          <t>진실한, 진심 어린</t>
+        </is>
+      </c>
+      <c r="Y146" s="9" t="inlineStr">
+        <is>
+          <t>로마 조각가가 결함을 밀랍으로 숨겼는데, 최고 작품은 밀랍 없이(sine cera) 완성됨</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>